<commit_message>
Update Excel data file for certificate generation
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="24980" windowHeight="13060"/>
+    <workbookView windowWidth="29400" windowHeight="14020"/>
   </bookViews>
   <sheets>
     <sheet name="Certificates" sheetId="2" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="207">
   <si>
     <t>Paper ID</t>
   </si>
@@ -139,7 +139,14 @@
     <t>Dr. Sumit Nema</t>
   </si>
   <si>
+    <t xml:space="preserve">Associate Professor, Computer Science and Engineering, Gyan Ganga Institute of Technology and Science, Jabalpur 
+</t>
+  </si>
+  <si>
     <t>Khushbu Kesharwani</t>
+  </si>
+  <si>
+    <t>St Aloysius College Autonomous, Jabalpur, India</t>
   </si>
   <si>
     <t>Richa Tiwari</t>
@@ -689,17 +696,10 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -722,13 +722,6 @@
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -875,7 +868,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -999,12 +992,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1199,19 +1186,28 @@
   </borders>
   <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1220,127 +1216,118 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
@@ -1352,22 +1339,22 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="49" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="49" applyBorder="1" applyAlignment="1">
@@ -1970,7 +1957,7 @@
         <v>31</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" ht="44" spans="1:4">
@@ -1981,10 +1968,10 @@
         <v>26</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20" ht="44" spans="1:4">
@@ -1995,7 +1982,7 @@
         <v>26</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>28</v>
@@ -2006,13 +1993,13 @@
         <v>125</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" ht="29" spans="1:4">
@@ -2020,13 +2007,13 @@
         <v>125</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" ht="29" spans="1:4">
@@ -2034,13 +2021,13 @@
         <v>125</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C23" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D23" s="6" t="s">
         <v>38</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="24" ht="29" spans="1:4">
@@ -2048,13 +2035,13 @@
         <v>146</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="25" ht="29" spans="1:4">
@@ -2062,13 +2049,13 @@
         <v>146</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="26" ht="29" spans="1:4">
@@ -2076,13 +2063,13 @@
         <v>146</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C26" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="D26" s="6" t="s">
         <v>43</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="27" ht="29" spans="1:4">
@@ -2090,13 +2077,13 @@
         <v>146</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="28" ht="58" spans="1:4">
@@ -2104,13 +2091,13 @@
         <v>172</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="29" ht="58" spans="1:4">
@@ -2118,13 +2105,13 @@
         <v>172</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="30" ht="58" spans="1:4">
@@ -2132,13 +2119,13 @@
         <v>172</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="31" ht="58" spans="1:4">
@@ -2146,13 +2133,13 @@
         <v>172</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C31" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="D31" s="6" t="s">
         <v>51</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="32" ht="29" spans="1:4">
@@ -2160,13 +2147,13 @@
         <v>220</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="33" ht="29" spans="1:4">
@@ -2174,13 +2161,13 @@
         <v>220</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="34" ht="58" spans="1:4">
@@ -2188,13 +2175,13 @@
         <v>223</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="35" ht="58" spans="1:4">
@@ -2202,13 +2189,13 @@
         <v>223</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="36" ht="58" spans="1:4">
@@ -2216,13 +2203,13 @@
         <v>223</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="37" ht="58" spans="1:4">
@@ -2230,13 +2217,13 @@
         <v>223</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="38" ht="44" spans="1:4">
@@ -2244,13 +2231,13 @@
         <v>267</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D38" s="10" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="39" ht="44" spans="1:4">
@@ -2258,13 +2245,13 @@
         <v>267</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="40" ht="44" spans="1:4">
@@ -2272,13 +2259,13 @@
         <v>267</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C40" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="D40" s="10" t="s">
         <v>67</v>
-      </c>
-      <c r="D40" s="10" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="41" ht="44" spans="1:4">
@@ -2286,13 +2273,13 @@
         <v>271</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="42" ht="44" spans="1:4">
@@ -2300,13 +2287,13 @@
         <v>271</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="43" ht="29" spans="1:4">
@@ -2314,13 +2301,13 @@
         <v>276</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C43" s="10" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="44" ht="29" spans="1:4">
@@ -2328,13 +2315,13 @@
         <v>276</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D44" s="10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="45" ht="29" spans="1:4">
@@ -2342,13 +2329,13 @@
         <v>276</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="46" ht="29" spans="1:4">
@@ -2356,13 +2343,13 @@
         <v>276</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="47" ht="29" spans="1:4">
@@ -2370,13 +2357,13 @@
         <v>276</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="48" ht="29" spans="1:4">
@@ -2384,13 +2371,13 @@
         <v>276</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C48" s="10" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D48" s="10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="49" ht="29" spans="1:4">
@@ -2398,13 +2385,13 @@
         <v>279</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C49" s="10" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D49" s="10" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="50" ht="29" spans="1:4">
@@ -2412,13 +2399,13 @@
         <v>279</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C50" s="10" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D50" s="10" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="51" ht="29" spans="1:4">
@@ -2426,13 +2413,13 @@
         <v>291</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C51" s="10" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="52" ht="29" spans="1:4">
@@ -2440,13 +2427,13 @@
         <v>291</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C52" s="10" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="53" ht="58" spans="1:4">
@@ -2454,13 +2441,13 @@
         <v>293</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="54" ht="58" spans="1:4">
@@ -2468,13 +2455,13 @@
         <v>293</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="55" ht="58" spans="1:4">
@@ -2482,13 +2469,13 @@
         <v>293</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C55" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D55" s="6" t="s">
         <v>96</v>
-      </c>
-      <c r="D55" s="6" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="56" ht="44" spans="1:4">
@@ -2496,13 +2483,13 @@
         <v>304</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="57" ht="44" spans="1:4">
@@ -2510,13 +2497,13 @@
         <v>304</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="58" ht="29" spans="1:4">
@@ -2524,13 +2511,13 @@
         <v>306</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="59" ht="29" spans="1:4">
@@ -2538,13 +2525,13 @@
         <v>306</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C59" s="10" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="60" ht="29" spans="1:4">
@@ -2552,13 +2539,13 @@
         <v>306</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C60" s="10" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="61" ht="29" spans="1:4">
@@ -2566,13 +2553,13 @@
         <v>309</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C61" s="10" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D61" s="10" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="62" ht="29" spans="1:4">
@@ -2580,13 +2567,13 @@
         <v>309</v>
       </c>
       <c r="B62" s="10" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C62" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D62" s="10" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="63" ht="44" spans="1:4">
@@ -2594,13 +2581,13 @@
         <v>317</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C63" s="10" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D63" s="10" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="64" ht="44" spans="1:4">
@@ -2608,13 +2595,13 @@
         <v>317</v>
       </c>
       <c r="B64" s="10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C64" s="10" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D64" s="10" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="65" ht="44" spans="1:4">
@@ -2622,13 +2609,13 @@
         <v>317</v>
       </c>
       <c r="B65" s="10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C65" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="D65" s="10" t="s">
         <v>113</v>
-      </c>
-      <c r="D65" s="10" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="66" ht="44" spans="1:4">
@@ -2636,13 +2623,13 @@
         <v>317</v>
       </c>
       <c r="B66" s="10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C66" s="10" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D66" s="10" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="67" ht="44" spans="1:4">
@@ -2650,13 +2637,13 @@
         <v>317</v>
       </c>
       <c r="B67" s="10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C67" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D67" s="10" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="68" ht="44" spans="1:4">
@@ -2664,13 +2651,13 @@
         <v>317</v>
       </c>
       <c r="B68" s="10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C68" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D68" s="10" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="69" ht="44" spans="1:4">
@@ -2678,13 +2665,13 @@
         <v>332</v>
       </c>
       <c r="B69" s="10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C69" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D69" s="10" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="70" ht="44" spans="1:4">
@@ -2692,13 +2679,13 @@
         <v>332</v>
       </c>
       <c r="B70" s="10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C70" s="10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D70" s="10" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="71" ht="44" spans="1:4">
@@ -2706,13 +2693,13 @@
         <v>332</v>
       </c>
       <c r="B71" s="10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C71" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="D71" s="10" t="s">
         <v>121</v>
-      </c>
-      <c r="D71" s="10" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="72" ht="29" spans="1:4">
@@ -2720,13 +2707,13 @@
         <v>333</v>
       </c>
       <c r="B72" s="10" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C72" s="10" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D72" s="10" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="73" ht="29" spans="1:4">
@@ -2734,13 +2721,13 @@
         <v>333</v>
       </c>
       <c r="B73" s="10" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C73" s="10" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D73" s="10" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="74" ht="29" spans="1:4">
@@ -2748,13 +2735,13 @@
         <v>333</v>
       </c>
       <c r="B74" s="10" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C74" s="10" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D74" s="10" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="75" ht="29" spans="1:4">
@@ -2762,13 +2749,13 @@
         <v>333</v>
       </c>
       <c r="B75" s="10" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C75" s="10" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D75" s="10" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="76" ht="29" spans="1:4">
@@ -2776,13 +2763,13 @@
         <v>333</v>
       </c>
       <c r="B76" s="10" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C76" s="10" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D76" s="10" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="77" ht="29" spans="1:4">
@@ -2790,13 +2777,13 @@
         <v>336</v>
       </c>
       <c r="B77" s="10" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C77" s="10" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D77" s="10" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="78" ht="29" spans="1:4">
@@ -2804,13 +2791,13 @@
         <v>336</v>
       </c>
       <c r="B78" s="10" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C78" s="10" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D78" s="10" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="79" ht="29" spans="1:4">
@@ -2818,13 +2805,13 @@
         <v>336</v>
       </c>
       <c r="B79" s="10" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C79" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="D79" s="10" t="s">
         <v>136</v>
-      </c>
-      <c r="D79" s="10" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="80" ht="29" spans="1:4">
@@ -2832,13 +2819,13 @@
         <v>336</v>
       </c>
       <c r="B80" s="10" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C80" s="10" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D80" s="10" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="81" ht="29" spans="1:4">
@@ -2846,13 +2833,13 @@
         <v>336</v>
       </c>
       <c r="B81" s="10" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C81" s="10" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D81" s="10" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="82" ht="29" spans="1:4">
@@ -2860,13 +2847,13 @@
         <v>340</v>
       </c>
       <c r="B82" s="10" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C82" s="10" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D82" s="10" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="83" ht="29" spans="1:4">
@@ -2874,13 +2861,13 @@
         <v>340</v>
       </c>
       <c r="B83" s="10" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C83" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D83" s="10" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="84" ht="44" spans="1:4">
@@ -2888,13 +2875,13 @@
         <v>352</v>
       </c>
       <c r="B84" s="10" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C84" s="10" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="85" ht="44" spans="1:4">
@@ -2902,13 +2889,13 @@
         <v>352</v>
       </c>
       <c r="B85" s="10" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C85" s="10" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="86" ht="44" spans="1:4">
@@ -2916,13 +2903,13 @@
         <v>352</v>
       </c>
       <c r="B86" s="10" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C86" s="10" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="87" ht="44" spans="1:4">
@@ -2930,13 +2917,13 @@
         <v>354</v>
       </c>
       <c r="B87" s="10" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C87" s="10" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="88" ht="44" spans="1:4">
@@ -2944,13 +2931,13 @@
         <v>354</v>
       </c>
       <c r="B88" s="10" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C88" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="89" ht="29" spans="1:4">
@@ -2958,13 +2945,13 @@
         <v>355</v>
       </c>
       <c r="B89" s="10" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C89" s="10" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D89" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="90" ht="29" spans="1:4">
@@ -2972,13 +2959,13 @@
         <v>355</v>
       </c>
       <c r="B90" s="10" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C90" s="10" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="91" ht="29" spans="1:4">
@@ -2986,13 +2973,13 @@
         <v>355</v>
       </c>
       <c r="B91" s="10" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C91" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D91" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="92" ht="29" spans="1:4">
@@ -3000,13 +2987,13 @@
         <v>355</v>
       </c>
       <c r="B92" s="10" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C92" s="10" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D92" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="93" spans="1:4">
@@ -4869,145 +4856,145 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B1" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C1" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B2" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B3" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B4" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C4" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B5" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B6" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="1" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B7" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C7" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B8" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C8" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="1" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C9" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="1" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B10" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C10" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B11" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C11" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="1" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B12" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C12" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B13" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C13" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -5028,42 +5015,42 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -5080,27 +5067,27 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data.xlsx for certificate generation
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29400" windowHeight="14020"/>
+    <workbookView windowWidth="29400" windowHeight="12620" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Certificates" sheetId="2" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="208">
   <si>
     <t>Paper ID</t>
   </si>
@@ -669,6 +669,9 @@
   </si>
   <si>
     <t>Dr. Abhinav Pathak</t>
+  </si>
+  <si>
+    <t>Dr. Shweta Agrawal</t>
   </si>
   <si>
     <t>Karishma Parwani</t>
@@ -1379,7 +1382,7 @@
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -5010,8 +5013,8 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A8"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="7"/>
+  <dimension ref="A1:A9"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
@@ -5051,6 +5054,11 @@
     <row r="8" spans="1:1">
       <c r="A8" t="s">
         <v>201</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" t="s">
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -5067,27 +5075,27 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
   </sheetData>

</xml_diff>